<commit_message>
Use system Chrome directly - no remote debugging needed
</commit_message>
<xml_diff>
--- a/excel/HoaDon.xlsx
+++ b/excel/HoaDon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\duancongty\botmail\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2297687-3980-43B8-BA1F-0F72D322F915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDA7A53-4AF5-48ED-ADB1-991F264B1CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="137">
   <si>
     <t>ID hóa đơn</t>
   </si>
@@ -118,6 +118,177 @@
     <t>8109290301</t>
   </si>
   <si>
+    <t>SOBD37734297</t>
+  </si>
+  <si>
+    <t>20/05/2026 00:26:01</t>
+  </si>
+  <si>
+    <t>37734297.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Quầy thuốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QT Khiêm Việt Xà Bang </t>
+  </si>
+  <si>
+    <t>Khiêm việt</t>
+  </si>
+  <si>
+    <t>Tổ 18.ấp xà bang1.xã xà bang.châu đưc.ba ria vũng tàu</t>
+  </si>
+  <si>
+    <t>8829328799-001</t>
+  </si>
+  <si>
+    <t>SOBD37786453</t>
+  </si>
+  <si>
+    <t>20/05/2026 00:25:57</t>
+  </si>
+  <si>
+    <t>37786453.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>QT Hải Yến 10</t>
+  </si>
+  <si>
+    <t>Quầy thuốc Hải Yến 10</t>
+  </si>
+  <si>
+    <t>Tổ 28, Ấp 4, xã An phước, tỉnh Đồng Nai</t>
+  </si>
+  <si>
+    <t>3603807776</t>
+  </si>
+  <si>
+    <t>SOBD37745129</t>
+  </si>
+  <si>
+    <t>20/05/2026 01:46:05</t>
+  </si>
+  <si>
+    <t>37745129.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Nhà thuốc Anh Tiến</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH NHÀ THUỐC ANH TIẾN</t>
+  </si>
+  <si>
+    <t>Số 124, đường Đê bao, ấp 2-3, Xã Tân Vĩnh Lộc, TP Hồ Chí Minh</t>
+  </si>
+  <si>
+    <t>079097028014</t>
+  </si>
+  <si>
+    <t>SOBD37812149</t>
+  </si>
+  <si>
+    <t>20/05/2026 00:25:58</t>
+  </si>
+  <si>
+    <t>37812149.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Trần Thị Thúy (Thanh Thúy A 30)</t>
+  </si>
+  <si>
+    <t>Tổ 15, ấp Bến Sắn, Phường Nhơn Trạch, TP Đồng Nai</t>
+  </si>
+  <si>
+    <t>075190025400</t>
+  </si>
+  <si>
+    <t>SOHN37756340</t>
+  </si>
+  <si>
+    <t>27/05/2026 23:59:59</t>
+  </si>
+  <si>
+    <t>15/05/2026 10:19:48</t>
+  </si>
+  <si>
+    <t>37756340.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Quầy thuốc Hà Lành</t>
+  </si>
+  <si>
+    <t>quầy thuốc Hà Lành</t>
+  </si>
+  <si>
+    <t>ngã 3 Mẫu Sơn xã Khánh Xuân huyện Lộc Bình tỉnh Lạng Sơn</t>
+  </si>
+  <si>
+    <t>4900881284</t>
+  </si>
+  <si>
+    <t>SOHN37780110</t>
+  </si>
+  <si>
+    <t>19/05/2026 13:35:19</t>
+  </si>
+  <si>
+    <t>37780110.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Quầy Thuốc Phương Trâm</t>
+  </si>
+  <si>
+    <t>Quầy Thuốc  Phương Trâm</t>
+  </si>
+  <si>
+    <t>khu 3, Nội Đồng, Đại Thịnh,  Mê Linh, Hà Nội</t>
+  </si>
+  <si>
+    <t>8596170972</t>
+  </si>
+  <si>
+    <t>SOBD37815063</t>
+  </si>
+  <si>
+    <t>19/05/2026 00:25:46</t>
+  </si>
+  <si>
+    <t>37815063.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>QUẦY THUỐC NHÂN THẢO</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH QUẦY THUỐC NHÂN THẢO</t>
+  </si>
+  <si>
+    <t>Tổ 23, Khu C, ấp Phước Lý, Xã Đại Phước, TP Đồng Nai</t>
+  </si>
+  <si>
+    <t>075190020134</t>
+  </si>
+  <si>
+    <t>SOHN37809478</t>
+  </si>
+  <si>
+    <t>19/05/2026 06:52:20</t>
+  </si>
+  <si>
+    <t>37809478.Z2I4OQEM8D@hoadon.thuocsi.vn</t>
+  </si>
+  <si>
+    <t>Ngô Quỳnh Anh</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH QUẦY THUỐC BẠCH MAI PHARMACY 89</t>
+  </si>
+  <si>
+    <t>Thôn Xuân Tràng, Xã Hoàn Long, Hưng Yên</t>
+  </si>
+  <si>
+    <t>033301004213</t>
+  </si>
+  <si>
     <t>#</t>
   </si>
   <si>
@@ -239,6 +410,33 @@
   </si>
   <si>
     <t>https://sellercenter.thuocsi.vn/order/invoice/XAHY84FW</t>
+  </si>
+  <si>
+    <t>1TCQDBCV</t>
+  </si>
+  <si>
+    <t>20/05/2026 09:05:46</t>
+  </si>
+  <si>
+    <t>GOILANAU10</t>
+  </si>
+  <si>
+    <t>Gội là nâu thảo dược lucky star (h/10g/25ml)</t>
+  </si>
+  <si>
+    <t>[302604/010329/1]</t>
+  </si>
+  <si>
+    <t>https://sellercenter.thuocsi.vn/order/invoice/1TCQDBCV</t>
+  </si>
+  <si>
+    <t>[302602/020329/1]</t>
+  </si>
+  <si>
+    <t>Nguyễn Vũ Giang Bắc (Nhà Thuốc Phương Bắc)</t>
+  </si>
+  <si>
+    <t>2406 Huỳnh Tấn Phát, ấp 3, Xã Nhà Bè, TP Hồ Chí Minh, Việt Nam</t>
   </si>
 </sst>
 </file>
@@ -274,8 +472,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,14 +816,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="9" max="9" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="37.875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="48.875" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +868,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -723,7 +918,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>12811160</v>
       </c>
@@ -770,54 +965,400 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:16" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>12810193</v>
+      </c>
+      <c r="B4">
+        <v>37734297</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4">
+        <v>385000</v>
+      </c>
+      <c r="I4">
+        <v>385000</v>
+      </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>12806060</v>
+      </c>
+      <c r="B5">
+        <v>37786453</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5">
+        <v>130000</v>
+      </c>
+      <c r="I5">
+        <v>130000</v>
+      </c>
+      <c r="J5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" t="s">
+        <v>41</v>
+      </c>
+      <c r="N5" t="s">
+        <v>42</v>
+      </c>
+      <c r="O5" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>12801159</v>
+      </c>
+      <c r="B6">
+        <v>37745129</v>
+      </c>
+      <c r="C6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6">
+        <v>350000</v>
+      </c>
+      <c r="I6">
+        <v>350000</v>
+      </c>
+      <c r="J6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" t="s">
+        <v>50</v>
+      </c>
+      <c r="P6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>12799484</v>
+      </c>
+      <c r="B7">
+        <v>37812149</v>
+      </c>
+      <c r="C7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>52800</v>
+      </c>
+      <c r="I7">
+        <v>52800</v>
+      </c>
+      <c r="J7" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O7" t="s">
+        <v>56</v>
+      </c>
+      <c r="P7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>12796727</v>
+      </c>
+      <c r="B8">
+        <v>37756340</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8">
+        <v>75800</v>
+      </c>
+      <c r="I8">
+        <v>75800</v>
+      </c>
+      <c r="J8" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" t="s">
+        <v>62</v>
+      </c>
+      <c r="N8" t="s">
+        <v>63</v>
+      </c>
+      <c r="O8" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>12792938</v>
+      </c>
+      <c r="B9">
+        <v>37780110</v>
+      </c>
+      <c r="C9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9">
+        <v>46600</v>
+      </c>
+      <c r="I9">
+        <v>46600</v>
+      </c>
+      <c r="J9" t="s">
+        <v>68</v>
+      </c>
+      <c r="K9" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" t="s">
+        <v>69</v>
+      </c>
+      <c r="N9" t="s">
+        <v>70</v>
+      </c>
+      <c r="O9" t="s">
+        <v>71</v>
+      </c>
+      <c r="P9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>12788180</v>
+      </c>
+      <c r="B10">
+        <v>37815063</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10">
+        <v>175000</v>
+      </c>
+      <c r="I10">
+        <v>175000</v>
+      </c>
+      <c r="J10" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" t="s">
+        <v>33</v>
+      </c>
+      <c r="M10" t="s">
+        <v>76</v>
+      </c>
+      <c r="N10" t="s">
+        <v>77</v>
+      </c>
+      <c r="O10" t="s">
+        <v>78</v>
+      </c>
+      <c r="P10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>12784829</v>
+      </c>
+      <c r="B11">
+        <v>37809478</v>
+      </c>
+      <c r="C11" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11">
+        <v>106000</v>
+      </c>
+      <c r="I11">
+        <v>106000</v>
+      </c>
+      <c r="J11" t="s">
+        <v>82</v>
+      </c>
+      <c r="K11" t="s">
+        <v>25</v>
+      </c>
+      <c r="L11" t="s">
+        <v>33</v>
+      </c>
+      <c r="M11" t="s">
+        <v>83</v>
+      </c>
+      <c r="N11" t="s">
+        <v>84</v>
+      </c>
+      <c r="O11" t="s">
+        <v>85</v>
+      </c>
+      <c r="P11" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:P3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:P11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AK13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.75" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.75" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="24.75" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.75" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="47.75" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="37.875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="47.875" customWidth="1"/>
+    <col min="36" max="36" width="54.75" customWidth="1"/>
+    <col min="37" max="37" width="14.625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -826,13 +1367,13 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>89</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
@@ -844,67 +1385,67 @@
         <v>5</v>
       </c>
       <c r="J1" t="s">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="K1" t="s">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="L1" t="s">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="M1" t="s">
-        <v>36</v>
+        <v>93</v>
       </c>
       <c r="N1" t="s">
-        <v>37</v>
+        <v>94</v>
       </c>
       <c r="O1" t="s">
-        <v>38</v>
+        <v>95</v>
       </c>
       <c r="P1" t="s">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="Q1" t="s">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="R1" t="s">
-        <v>41</v>
+        <v>98</v>
       </c>
       <c r="S1" t="s">
-        <v>42</v>
+        <v>99</v>
       </c>
       <c r="T1" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="U1" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="V1" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
       <c r="W1" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
       <c r="X1" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="Y1" t="s">
         <v>8</v>
       </c>
       <c r="Z1" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
       <c r="AA1" t="s">
-        <v>49</v>
+        <v>106</v>
       </c>
       <c r="AB1" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
       <c r="AC1" t="s">
-        <v>51</v>
+        <v>108</v>
       </c>
       <c r="AD1" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="AE1" t="s">
         <v>9</v>
@@ -924,11 +1465,11 @@
       <c r="AJ1" t="s">
         <v>14</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -969,7 +1510,7 @@
         <v>16</v>
       </c>
       <c r="N2" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="O2" t="s">
         <v>17</v>
@@ -978,31 +1519,31 @@
         <v>18</v>
       </c>
       <c r="Q2" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="R2" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="S2" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
       <c r="T2" t="s">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="U2" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
       <c r="V2" t="s">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="W2" t="s">
-        <v>60</v>
+        <v>117</v>
       </c>
       <c r="X2" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
       <c r="Y2" t="s">
-        <v>62</v>
+        <v>119</v>
       </c>
       <c r="Z2" t="s">
         <v>16</v>
@@ -1037,11 +1578,11 @@
       <c r="AJ2" t="s">
         <v>16</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AK2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1052,13 +1593,13 @@
         <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="E3" t="s">
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>121</v>
       </c>
       <c r="G3">
         <v>37788276</v>
@@ -1070,16 +1611,16 @@
         <v>23</v>
       </c>
       <c r="J3" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="K3">
         <v>91712</v>
       </c>
       <c r="L3" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="N3">
         <v>175000</v>
@@ -1115,16 +1656,16 @@
         <v>175000</v>
       </c>
       <c r="Z3" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
       <c r="AA3" t="s">
-        <v>69</v>
+        <v>126</v>
       </c>
       <c r="AB3" t="s">
         <v>16</v>
       </c>
       <c r="AC3" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
       <c r="AE3" t="s">
         <v>24</v>
@@ -1139,32 +1680,238 @@
         <v>27</v>
       </c>
       <c r="AI3" t="s">
-        <v>27</v>
+        <v>135</v>
       </c>
       <c r="AJ3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AK3" t="s">
+        <v>136</v>
+      </c>
+      <c r="AK3" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:37" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>12801159</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4">
+        <v>37745129</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K4">
+        <v>91711</v>
+      </c>
+      <c r="L4" t="s">
+        <v>130</v>
+      </c>
+      <c r="M4" t="s">
+        <v>131</v>
+      </c>
+      <c r="N4">
+        <v>175000</v>
+      </c>
+      <c r="O4">
+        <v>173884</v>
+      </c>
+      <c r="P4">
+        <v>175000</v>
+      </c>
+      <c r="Q4">
+        <v>8</v>
+      </c>
+      <c r="R4">
+        <v>162037</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4">
+        <v>1</v>
+      </c>
+      <c r="U4">
+        <v>1</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
+      <c r="Y4">
+        <v>175000</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>125</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>132</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>12801159</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G5">
+        <v>37745129</v>
+      </c>
+      <c r="H5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" t="s">
+        <v>129</v>
+      </c>
+      <c r="K5">
+        <v>91712</v>
+      </c>
+      <c r="L5" t="s">
+        <v>123</v>
+      </c>
+      <c r="M5" t="s">
+        <v>124</v>
+      </c>
+      <c r="N5">
+        <v>175000</v>
+      </c>
+      <c r="O5">
+        <v>169118</v>
+      </c>
+      <c r="P5">
+        <v>175000</v>
+      </c>
+      <c r="Q5">
+        <v>8</v>
+      </c>
+      <c r="R5">
+        <v>162037</v>
+      </c>
+      <c r="S5">
+        <v>1</v>
+      </c>
+      <c r="T5">
+        <v>1</v>
+      </c>
+      <c r="U5">
+        <v>1</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
+      <c r="Y5">
+        <v>175000</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>125</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>134</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>50</v>
+      </c>
+      <c r="AK5" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="AC3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="AC4" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="AC5" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AK3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:AK2 A3:AH3 AK3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>